<commit_message>
Update soccer trades 2026-07-27 16:01:18 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/UEFA Conference League/trades.xlsx
+++ b/data/sxbet/ligas/UEFA Conference League/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V16"/>
+  <dimension ref="A1:V26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,59 +531,67 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xb86a834aa70af447f0675d386c1849b1c99fbb8415a4a0f57dedbfc3374369c8</t>
+          <t>0x00ae6c3a5ed7e25ed4adcc5d726b723762a6ddfb651274951dc984b567621eef</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
+          <t>0x40C6406af6250bDC2d12E0AA4053630789f332c2</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>10.74</t>
+          <t>1.819</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.2875</t>
+          <t>1.1675</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Dukagjini</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
           <t>UEFA Conference League</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>UEFA Conference League</t>
-        </is>
-      </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>KF Drita vs Floriana</t>
+          <t>Dukagjini vs FC Lugano</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>KF Drita</t>
+          <t>Dukagjini</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Floriana</t>
+          <t>FC Lugano</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x74cee3640eed67802d8602418d415d7e5f881528425b4aded0a73b883c57f7c2</t>
+          <t>0xb4e6b34f8bd841e610d92a6e94ae60f508da52a98987521a70ab1ff92547c4a1</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19556829</t>
+          <t>L19578699</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -608,17 +616,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785068425</t>
+          <t>1785164985</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1785261600</t>
+          <t>1785335400</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>37.356522</t>
+          <t>10.859701</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,12 +643,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x8004902c8df50fb0691955c2dde204aa37aea6ffc9f11cb60795a2b8862e7e34</t>
+          <t>0x3d30d13f4f7532b8458d9fcb5fefaa11b7fdc084e05b8ea5921efdd1815c2b2e</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+          <t>0x40C6406af6250bDC2d12E0AA4053630789f332c2</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -650,22 +658,22 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1.69</t>
+          <t>1.802</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.3188</t>
+          <t>1.1675</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>KF Drita -1.5</t>
+          <t>Dukagjini</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -675,27 +683,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>KF Drita vs Floriana</t>
+          <t>Dukagjini vs FC Lugano</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>KF Drita</t>
+          <t>Dukagjini</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Floriana</t>
+          <t>FC Lugano</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x9a6a1619c23e931d4f7a0e722354bdd7a98d7591c8e2ec98666a74ed9b164c2d</t>
+          <t>0xb4e6b34f8bd841e610d92a6e94ae60f508da52a98987521a70ab1ff92547c4a1</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19556829</t>
+          <t>L19578699</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -720,17 +728,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1785065693</t>
+          <t>1785162974</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1785261600</t>
+          <t>1785335400</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>5.301961</t>
+          <t>10.758209</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -747,39 +755,31 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x9d52e065d77a1e2ffa07fa7250522f55f6a20661ddb8ab22b3656a5e5f518751</t>
+          <t>0x79647a96f9215372245b4b53f196e63141ae86a1ea37ec3c520054924f339f07</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2.87</t>
+          <t>7.28</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.3188</t>
+          <t>1.2975</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>KF Drita -1.5</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>UEFA Conference League</t>
@@ -787,27 +787,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>KF Drita vs Floriana</t>
+          <t>Apollon Limassol FC vs FC Dila Gori</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>KF Drita</t>
+          <t>Apollon Limassol FC</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Floriana</t>
+          <t>FC Dila Gori</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x9a6a1619c23e931d4f7a0e722354bdd7a98d7591c8e2ec98666a74ed9b164c2d</t>
+          <t>0x000702f32390bc2acb841097855bbcf831db778647d8ef65ce0eb22695863bdc</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19556829</t>
+          <t>L19548403</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -832,17 +832,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1785065679</t>
+          <t>1785160034</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1785261600</t>
+          <t>1785258000</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>9.003922</t>
+          <t>24.470588</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -859,12 +859,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0xf072d053c048f056d7fa49c75da51e0772df0db003eaf3ddf341cb2fcc16c416</t>
+          <t>0xc738fb5ab6b1a30b7c6c1ec2cd7f70095001f6e7c404f7f168998f3ce0923565</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+          <t>0x0fE55cE066A9810115Ea99B11a14e96a4b635810</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -874,22 +874,22 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>281.53996</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.3188</t>
+          <t>1.8588</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>UEFA Conference League</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>KF Drita -1.5</t>
+          <t>Apollon Limassol FC</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -899,27 +899,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>KF Drita vs Floriana</t>
+          <t>Apollon Limassol FC vs FC Dila Gori</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>KF Drita</t>
+          <t>Apollon Limassol FC</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Floriana</t>
+          <t>FC Dila Gori</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0x9a6a1619c23e931d4f7a0e722354bdd7a98d7591c8e2ec98666a74ed9b164c2d</t>
+          <t>0x6b053f472a4306388af8fe5ea15275295a0aae1b19a9f51e5b3c924cb4aacd4d</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>L19556829</t>
+          <t>L19548403</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -944,17 +944,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1785065519</t>
+          <t>1785159837</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>1785261600</t>
+          <t>1785258000</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>14.117647</t>
+          <t>327.848571</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -971,7 +971,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0xe1a18ecff833fc919588fdf2e22421fae16e5d31600f43cd14887e49499b233e</t>
+          <t>0x0b99d0d305609060f8495bfe5f8c95e1a0b399ad11cc9adf4f34153f68c97d71</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -986,22 +986,22 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>3.01</t>
+          <t>1.01</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.3325</t>
+          <t>1.1025</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>KF Drita -1.5</t>
+          <t>FC Dila Gori</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1011,27 +1011,27 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>KF Drita vs Floriana</t>
+          <t>Apollon Limassol FC vs FC Dila Gori</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>KF Drita</t>
+          <t>Apollon Limassol FC</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Floriana</t>
+          <t>FC Dila Gori</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0x9a6a1619c23e931d4f7a0e722354bdd7a98d7591c8e2ec98666a74ed9b164c2d</t>
+          <t>0x66b17a5927b2a92224c605c32e8306f8dc8fabb6ccff81abfc5fbafb709f9a22</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>L19556829</t>
+          <t>L19548403</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1056,17 +1056,17 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1785065131</t>
+          <t>1785143243</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>1785261600</t>
+          <t>1785258000</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>9.052632</t>
+          <t>9.853659</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1083,12 +1083,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x97e956b7b7cfe7d56ae2e8711191f397ae89244a032e763798c4b0021c72d481</t>
+          <t>0xa2274ee0f4684479f0988ac6a5139708014cf026476c7cf9b37b3a416e7b5747</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+          <t>0x1b1185C2A2d1Ec3CA592f5c21f52dD4aD449163f</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1098,22 +1098,22 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3.81</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.3325</t>
+          <t>1.0625</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>KF Drita -1.5</t>
+          <t>Paide Linnameeskond</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1123,27 +1123,27 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>KF Drita vs Floriana</t>
+          <t>Zira FK vs Paide Linnameeskond</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>KF Drita</t>
+          <t>Zira FK</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Floriana</t>
+          <t>Paide Linnameeskond</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x9a6a1619c23e931d4f7a0e722354bdd7a98d7591c8e2ec98666a74ed9b164c2d</t>
+          <t>0xc2274f3d5306fe3b7bf272b7cfce16894bf01595fd8fa3181858809c5afd887d</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>L19556829</t>
+          <t>L19568228</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1168,17 +1168,17 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1785065030</t>
+          <t>1785123628</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>1785261600</t>
+          <t>1785427200</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>11.458647</t>
+          <t>96.0</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1195,7 +1195,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x1b6d50b0b2f30b843c8afcdf1bdd77c807787389b518c0d0118f66c5c53154d1</t>
+          <t>0x4b249266f4a129a90a4f4289f80efd22864a0b55a615a30c01a744c9e6fa007e</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1210,22 +1210,22 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4.93</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.3325</t>
+          <t>1.2463</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>KF Drita -1.5</t>
+          <t>FC Spartak Trnava</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1235,27 +1235,27 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>KF Drita vs Floriana</t>
+          <t>FC CSKA Sofia 1948 vs FC Spartak Trnava</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>KF Drita</t>
+          <t>FC CSKA Sofia 1948</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Floriana</t>
+          <t>FC Spartak Trnava</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x9a6a1619c23e931d4f7a0e722354bdd7a98d7591c8e2ec98666a74ed9b164c2d</t>
+          <t>0xe6d3ed6a25306fb2793f56682ed261dbde83f239772758b37aeecc6a973830a6</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>L19556829</t>
+          <t>L19548391</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1280,17 +1280,17 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1785064974</t>
+          <t>1785114331</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>1785261600</t>
+          <t>1785259800</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>3.007519</t>
+          <t>20.020305</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1307,27 +1307,23 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0x7de08a0243073e49c6e479dead7f166232ecd3480830513fb8953abf4d30f575</t>
+          <t>0xbcaacd1e8dc7d60abd70f28c7ffba7450e4c76519b53d45633047b2e308ce8df</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x44cE278A4b373d2bFD26e6a2F5fA4E3550151d67</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.09</t>
+          <t>1.835</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1335,11 +1331,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Vardar</t>
-        </is>
-      </c>
+      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>UEFA Conference League</t>
@@ -1347,27 +1339,27 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Riga FC vs Vardar</t>
+          <t>Dukagjini vs FC Lugano</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Riga FC</t>
+          <t>Dukagjini</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Vardar</t>
+          <t>FC Lugano</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0x3df545e9e324274c452d3611c5ff53dc80c8487fce47da81056d17c1b4257d63</t>
+          <t>0xb4e6b34f8bd841e610d92a6e94ae60f508da52a98987521a70ab1ff92547c4a1</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>L19548393</t>
+          <t>L19578699</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1392,17 +1384,17 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1785064838</t>
+          <t>1785108140</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>1785258000</t>
+          <t>1785335400</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>13.333333</t>
+          <t>5.02994</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1419,28 +1411,28 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0x98d07c005cea52102549964e374db87ed764bdb1840c7e4d0822a34701829208</t>
+          <t>0xc4f834cac0960a0d1d3dfd961f4ed03d26a908325b0613bbc25d8271e7ea9596</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>11.17999</t>
+          <t>16.9</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.5012</t>
+          <t>1.4062</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
@@ -1451,27 +1443,27 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Riga FC vs Vardar</t>
+          <t>KF Drita vs Floriana</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Riga FC</t>
+          <t>KF Drita</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Vardar</t>
+          <t>Floriana</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0x3ce984b8d5a4fd077770e33c33bd5244077e868cb901d0b9544238e72630158d</t>
+          <t>0xd80db7f29b1a9bf7479fe759db5892459ba76d2573c8028c682ca72ca26fa563</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>L19548393</t>
+          <t>L19556829</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1496,17 +1488,17 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1785064821</t>
+          <t>1785102921</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>1785258000</t>
+          <t>1785261600</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>22.304219</t>
+          <t>41.6</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1523,12 +1515,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0x90084d34df7f1c1dba6533a65ec3b370264b980f4ee2f405409784667aef3385</t>
+          <t>0x642cead4cce6abf15e60b5f101292963653928af192a53d61cf13be1f5735346</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1538,22 +1530,22 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>13.33</t>
+          <t>25.11</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.34</t>
+          <t>1.485</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Asian Handicap (-2.5)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>KF Drita -1.5</t>
+          <t>SK Rapid Wien -2.5</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1563,27 +1555,27 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>KF Drita vs Floriana</t>
+          <t>SK Rapid Wien vs FC Santa Coloma</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>KF Drita</t>
+          <t>SK Rapid Wien</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Floriana</t>
+          <t>FC Santa Coloma</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0x9a6a1619c23e931d4f7a0e722354bdd7a98d7591c8e2ec98666a74ed9b164c2d</t>
+          <t>0x568429d159b17f3e17f83384554dcb4508d96942d411a493bfcdd9af2fd2df07</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>L19556829</t>
+          <t>L19558557</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1608,17 +1600,17 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1785064821</t>
+          <t>1785100795</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>1785261600</t>
+          <t>1785349800</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>39.205882</t>
+          <t>51.773196</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1635,39 +1627,31 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0xd382b16331a33a8ef623d9f672b5567e3faaf5a8c56a6b1abbd17c5b3bf2447a</t>
+          <t>0xb86a834aa70af447f0675d386c1849b1c99fbb8415a4a0f57dedbfc3374369c8</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1.25</t>
+          <t>10.74</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.09</t>
+          <t>1.2875</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Vardar</t>
-        </is>
-      </c>
+          <t>UEFA Conference League</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>UEFA Conference League</t>
@@ -1675,27 +1659,27 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Riga FC vs Vardar</t>
+          <t>KF Drita vs Floriana</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Riga FC</t>
+          <t>KF Drita</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Vardar</t>
+          <t>Floriana</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0x3df545e9e324274c452d3611c5ff53dc80c8487fce47da81056d17c1b4257d63</t>
+          <t>0x74cee3640eed67802d8602418d415d7e5f881528425b4aded0a73b883c57f7c2</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>L19548393</t>
+          <t>L19556829</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1720,17 +1704,17 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1785064819</t>
+          <t>1785068425</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>1785258000</t>
+          <t>1785261600</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>13.888889</t>
+          <t>37.356522</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1747,31 +1731,39 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0xc5ab66578686247686091622e73b8f1713617d5de6c2687bbf706bdd9a1c79eb</t>
+          <t>0x8004902c8df50fb0691955c2dde204aa37aea6ffc9f11cb60795a2b8862e7e34</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0x594542a29FFceEAeaDD2e67955437c928B51B758</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr"/>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>4.12</t>
+          <t>1.69</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.2637</t>
+          <t>1.3188</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr"/>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>KF Drita -1.5</t>
+        </is>
+      </c>
       <c r="H13" t="inlineStr">
         <is>
           <t>UEFA Conference League</t>
@@ -1779,27 +1771,27 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Riga FC vs Vardar</t>
+          <t>KF Drita vs Floriana</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Riga FC</t>
+          <t>KF Drita</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Vardar</t>
+          <t>Floriana</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0x8f444d513fee4c89c59a5fac9732f2bdbc34c255f1e145e912b5e8d3864de79a</t>
+          <t>0x9a6a1619c23e931d4f7a0e722354bdd7a98d7591c8e2ec98666a74ed9b164c2d</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>L19548393</t>
+          <t>L19556829</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1824,17 +1816,17 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1785064813</t>
+          <t>1785065693</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>1785258000</t>
+          <t>1785261600</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>15.620853</t>
+          <t>5.301961</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1851,7 +1843,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0x60648f843dfab3db80e7b11dc76bd422fb1242bf53219948830cbe4d1b29ee2e</t>
+          <t>0x9d52e065d77a1e2ffa07fa7250522f55f6a20661ddb8ab22b3656a5e5f518751</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1866,22 +1858,22 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>1.39</t>
+          <t>2.87</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.09</t>
+          <t>1.3188</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Vardar</t>
+          <t>KF Drita -1.5</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1891,27 +1883,27 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Riga FC vs Vardar</t>
+          <t>KF Drita vs Floriana</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Riga FC</t>
+          <t>KF Drita</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Vardar</t>
+          <t>Floriana</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0x3df545e9e324274c452d3611c5ff53dc80c8487fce47da81056d17c1b4257d63</t>
+          <t>0x9a6a1619c23e931d4f7a0e722354bdd7a98d7591c8e2ec98666a74ed9b164c2d</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>L19548393</t>
+          <t>L19556829</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1936,17 +1928,17 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1785064792</t>
+          <t>1785065679</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>1785258000</t>
+          <t>1785261600</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>15.444444</t>
+          <t>9.003922</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1963,31 +1955,39 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0xd4092c9aa9c679f18a84f2d088ee1a8595762c53fd62d16b214a853eff1fde81</t>
+          <t>0xf072d053c048f056d7fa49c75da51e0772df0db003eaf3ddf341cb2fcc16c416</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0x594542a29FFceEAeaDD2e67955437c928B51B758</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr"/>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>3.67</t>
+          <t>4.5</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.2637</t>
+          <t>1.3188</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr"/>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>KF Drita -1.5</t>
+        </is>
+      </c>
       <c r="H15" t="inlineStr">
         <is>
           <t>UEFA Conference League</t>
@@ -1995,27 +1995,27 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Riga FC vs Vardar</t>
+          <t>KF Drita vs Floriana</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Riga FC</t>
+          <t>KF Drita</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Vardar</t>
+          <t>Floriana</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0x8f444d513fee4c89c59a5fac9732f2bdbc34c255f1e145e912b5e8d3864de79a</t>
+          <t>0x9a6a1619c23e931d4f7a0e722354bdd7a98d7591c8e2ec98666a74ed9b164c2d</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>L19548393</t>
+          <t>L19556829</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -2040,17 +2040,17 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1785064770</t>
+          <t>1785065519</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>1785258000</t>
+          <t>1785261600</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>13.914692</t>
+          <t>14.117647</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2067,102 +2067,1198 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>0xe1a18ecff833fc919588fdf2e22421fae16e5d31600f43cd14887e49499b233e</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>3.01</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>1.3325</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>KF Drita -1.5</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>UEFA Conference League</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>KF Drita vs Floriana</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>KF Drita</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Floriana</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>0x9a6a1619c23e931d4f7a0e722354bdd7a98d7591c8e2ec98666a74ed9b164c2d</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>L19556829</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>1785065131</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>1785261600</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>9.052632</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>0x97e956b7b7cfe7d56ae2e8711191f397ae89244a032e763798c4b0021c72d481</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>3.81</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>1.3325</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>KF Drita -1.5</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>UEFA Conference League</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>KF Drita vs Floriana</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>KF Drita</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Floriana</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>0x9a6a1619c23e931d4f7a0e722354bdd7a98d7591c8e2ec98666a74ed9b164c2d</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>L19556829</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>1785065030</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>1785261600</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>11.458647</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>0x1b6d50b0b2f30b843c8afcdf1bdd77c807787389b518c0d0118f66c5c53154d1</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>1.3325</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>KF Drita -1.5</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>UEFA Conference League</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>KF Drita vs Floriana</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>KF Drita</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Floriana</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>0x9a6a1619c23e931d4f7a0e722354bdd7a98d7591c8e2ec98666a74ed9b164c2d</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>L19556829</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>1785064974</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>1785261600</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>3.007519</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>0x7de08a0243073e49c6e479dead7f166232ecd3480830513fb8953abf4d30f575</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>1.09</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Vardar</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>UEFA Conference League</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Riga FC vs Vardar</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Riga FC</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Vardar</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>0x3df545e9e324274c452d3611c5ff53dc80c8487fce47da81056d17c1b4257d63</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>L19548393</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>1785064838</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>1785258000</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>13.333333</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>0x98d07c005cea52102549964e374db87ed764bdb1840c7e4d0822a34701829208</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>11.17999</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>1.5012</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>UEFA Conference League</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Riga FC vs Vardar</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Riga FC</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Vardar</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>0x3ce984b8d5a4fd077770e33c33bd5244077e868cb901d0b9544238e72630158d</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>L19548393</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>1785064821</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>1785258000</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>22.304219</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>0x90084d34df7f1c1dba6533a65ec3b370264b980f4ee2f405409784667aef3385</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>13.33</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>1.34</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>KF Drita -1.5</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>UEFA Conference League</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>KF Drita vs Floriana</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>KF Drita</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Floriana</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>0x9a6a1619c23e931d4f7a0e722354bdd7a98d7591c8e2ec98666a74ed9b164c2d</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>L19556829</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>1785064821</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>1785261600</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>39.205882</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>0xd382b16331a33a8ef623d9f672b5567e3faaf5a8c56a6b1abbd17c5b3bf2447a</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>1.25</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>1.09</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Vardar</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>UEFA Conference League</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Riga FC vs Vardar</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Riga FC</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Vardar</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>0x3df545e9e324274c452d3611c5ff53dc80c8487fce47da81056d17c1b4257d63</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>L19548393</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>1785064819</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>1785258000</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>13.888889</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>0xc5ab66578686247686091622e73b8f1713617d5de6c2687bbf706bdd9a1c79eb</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>0x594542a29FFceEAeaDD2e67955437c928B51B758</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>4.12</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>1.2637</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>UEFA Conference League</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Riga FC vs Vardar</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Riga FC</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Vardar</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>0x8f444d513fee4c89c59a5fac9732f2bdbc34c255f1e145e912b5e8d3864de79a</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>L19548393</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>1785064813</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>1785258000</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>15.620853</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>0x60648f843dfab3db80e7b11dc76bd422fb1242bf53219948830cbe4d1b29ee2e</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>1.39</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>1.09</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Vardar</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>UEFA Conference League</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Riga FC vs Vardar</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Riga FC</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Vardar</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>0x3df545e9e324274c452d3611c5ff53dc80c8487fce47da81056d17c1b4257d63</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>L19548393</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>1785064792</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>1785258000</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>15.444444</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>0xd4092c9aa9c679f18a84f2d088ee1a8595762c53fd62d16b214a853eff1fde81</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>0x594542a29FFceEAeaDD2e67955437c928B51B758</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>3.67</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>1.2637</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>UEFA Conference League</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Riga FC vs Vardar</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Riga FC</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Vardar</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>0x8f444d513fee4c89c59a5fac9732f2bdbc34c255f1e145e912b5e8d3864de79a</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>L19548393</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>1785064770</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>1785258000</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>13.914692</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
           <t>0x3a9ab01f5b98d3619f0b7d9da475c1eabc0e13099a65941bdca6bd024e7991b6</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>0x44cE278A4b373d2bFD26e6a2F5fA4E3550151d67</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr">
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr">
         <is>
           <t>1.35</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>1.2637</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F26" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr">
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr">
         <is>
           <t>UEFA Conference League</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="I26" t="inlineStr">
         <is>
           <t>Riga FC vs Vardar</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="J26" t="inlineStr">
         <is>
           <t>Riga FC</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="K26" t="inlineStr">
         <is>
           <t>Vardar</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
+      <c r="L26" t="inlineStr">
         <is>
           <t>0x8f444d513fee4c89c59a5fac9732f2bdbc34c255f1e145e912b5e8d3864de79a</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
+      <c r="M26" t="inlineStr">
         <is>
           <t>L19548393</t>
         </is>
       </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P16" t="inlineStr">
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R16" t="inlineStr">
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
         <is>
           <t>1785064754</t>
         </is>
       </c>
-      <c r="S16" t="inlineStr">
+      <c r="S26" t="inlineStr">
         <is>
           <t>1785258000</t>
         </is>
       </c>
-      <c r="T16" t="inlineStr">
+      <c r="T26" t="inlineStr">
         <is>
           <t>5.118483</t>
         </is>
       </c>
-      <c r="U16" t="inlineStr">
+      <c r="U26" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V16" t="inlineStr">
+      <c r="V26" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>